<commit_message>
Started to trim Ethics1 down for GDV4000 Wk6. Adjusted groups for Explore
</commit_message>
<xml_diff>
--- a/T2/Explore_Groups_IS.xlsx
+++ b/T2/Explore_Groups_IS.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Ian\TEACHING_25_26\2025_26\T2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C2B74C8F-306A-4BD8-A143-55280851E887}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B740E6FA-AA6F-4B2D-80C2-E2C1B6C41E20}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="82440" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{B6CA3B6D-9BC0-410B-B5C1-C8E93D28BC64}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="27">
   <si>
     <t>Explore T2 Teams</t>
   </si>
@@ -114,6 +114,9 @@
   </si>
   <si>
     <t>Omreto</t>
+  </si>
+  <si>
+    <t>Muntasir Habib</t>
   </si>
 </sst>
 </file>
@@ -137,7 +140,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -174,6 +177,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -187,7 +196,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -202,6 +211,8 @@
     <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -536,7 +547,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DF8B7460-0B88-4778-815B-1377CD523625}">
-  <dimension ref="A1:B28"/>
+  <dimension ref="A1:B30"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="22.5703125" customWidth="1"/>
@@ -609,144 +620,159 @@
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A11" s="4" t="s">
+      <c r="A11" s="13" t="s">
+        <v>6</v>
+      </c>
+      <c r="B11" s="12"/>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A12" s="12" t="s">
         <v>9</v>
       </c>
-      <c r="B11" s="4">
+      <c r="B12" s="12">
         <v>20346949</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A12" s="4" t="s">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A13" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="B13" s="12">
+        <v>20347704</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A14" s="12" t="s">
         <v>10</v>
       </c>
-      <c r="B12" s="4">
+      <c r="B14" s="12">
         <v>20347202</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A13" s="7" t="s">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A15" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="B13" s="6"/>
-    </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A14" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="B14" s="6">
-        <v>20347506</v>
-      </c>
-    </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A15" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="B15" s="6">
-        <v>20346948</v>
-      </c>
+      <c r="B15" s="6"/>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" s="6" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B16" s="6">
-        <v>20346801</v>
+        <v>20347506</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="B17" s="6">
+        <v>20346948</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A18" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="B18" s="6">
+        <v>20346801</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A19" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="B17" s="6">
+      <c r="B19" s="6">
         <v>20351822</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A18" s="9" t="s">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A20" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="B18" s="8"/>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A19" s="8" t="s">
-        <v>16</v>
-      </c>
-      <c r="B19" s="8">
-        <v>20347352</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A20" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="B20" s="8">
-        <v>20347856</v>
-      </c>
+      <c r="B20" s="8"/>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" s="8" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="B21" s="8">
-        <v>20346739</v>
+        <v>20347352</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="B22" s="8">
+        <v>20347856</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A23" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="B23" s="8">
+        <v>20346739</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A24" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="B22" s="8">
+      <c r="B24" s="8">
         <v>20344884</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A23" s="11" t="s">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A25" s="11" t="s">
         <v>20</v>
       </c>
-      <c r="B23" s="10"/>
-    </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A24" s="10" t="s">
-        <v>21</v>
-      </c>
-      <c r="B24" s="10">
-        <v>20343328</v>
-      </c>
-    </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A25" s="10" t="s">
-        <v>22</v>
-      </c>
-      <c r="B25" s="10">
-        <v>20349661</v>
-      </c>
+      <c r="B25" s="10"/>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A26" s="10" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B26" s="10">
-        <v>20346858</v>
+        <v>20343328</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A27" s="10" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="B27" s="10">
-        <v>20344092</v>
+        <v>20349661</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A28" s="10" t="s">
+        <v>23</v>
+      </c>
+      <c r="B28" s="10">
+        <v>20346858</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A29" s="10" t="s">
+        <v>24</v>
+      </c>
+      <c r="B29" s="10">
+        <v>20344092</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A30" s="10" t="s">
         <v>25</v>
       </c>
-      <c r="B28" s="10">
+      <c r="B30" s="10">
         <v>20347355</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Updated groups for GDV4000 and Explore
</commit_message>
<xml_diff>
--- a/T2/Explore_Groups_IS.xlsx
+++ b/T2/Explore_Groups_IS.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Ian\TEACHING_25_26\2025_26\T2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B740E6FA-AA6F-4B2D-80C2-E2C1B6C41E20}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{72854A2A-4BFA-4898-B5AC-C681B7DD3E5F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="82440" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{B6CA3B6D-9BC0-410B-B5C1-C8E93D28BC64}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="28">
   <si>
     <t>Explore T2 Teams</t>
   </si>
@@ -117,6 +117,9 @@
   </si>
   <si>
     <t>Muntasir Habib</t>
+  </si>
+  <si>
+    <t>Labib Hasan</t>
   </si>
 </sst>
 </file>
@@ -140,7 +143,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -180,6 +183,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="5" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -196,7 +205,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -213,6 +222,7 @@
     <xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -547,7 +557,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DF8B7460-0B88-4778-815B-1377CD523625}">
-  <dimension ref="A1:B30"/>
+  <dimension ref="A1:B31"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="22.5703125" customWidth="1"/>
@@ -673,101 +683,109 @@
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" s="6" t="s">
-        <v>14</v>
+        <v>27</v>
       </c>
       <c r="B18" s="6">
-        <v>20346801</v>
+        <v>20347354</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="B19" s="6">
+        <v>20346801</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A20" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="B19" s="6">
+      <c r="B20" s="14">
         <v>20351822</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A20" s="9" t="s">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A21" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="B20" s="8"/>
-    </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A21" s="8" t="s">
-        <v>16</v>
-      </c>
-      <c r="B21" s="8">
-        <v>20347352</v>
-      </c>
+      <c r="B21" s="8"/>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" s="8" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B22" s="8">
-        <v>20347856</v>
+        <v>20347352</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23" s="8" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B23" s="8">
-        <v>20346739</v>
+        <v>20347856</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="B24" s="8">
+        <v>20346739</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A25" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="B24" s="8">
+      <c r="B25" s="8">
         <v>20344884</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A25" s="11" t="s">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A26" s="11" t="s">
         <v>20</v>
       </c>
-      <c r="B25" s="10"/>
-    </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A26" s="10" t="s">
-        <v>21</v>
-      </c>
-      <c r="B26" s="10">
-        <v>20343328</v>
-      </c>
+      <c r="B26" s="10"/>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A27" s="10" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B27" s="10">
-        <v>20349661</v>
+        <v>20343328</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A28" s="10" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B28" s="10">
-        <v>20346858</v>
+        <v>20349661</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A29" s="10" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B29" s="10">
-        <v>20344092</v>
+        <v>20346858</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A30" s="10" t="s">
+        <v>24</v>
+      </c>
+      <c r="B30" s="10">
+        <v>20344092</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A31" s="10" t="s">
         <v>25</v>
       </c>
-      <c r="B30" s="10">
+      <c r="B31" s="10">
         <v>20347355</v>
       </c>
     </row>

</xml_diff>